<commit_message>
Update Ibis Jaipur price history
</commit_message>
<xml_diff>
--- a/Accor_Ibis_Jaipur_Price_History.xlsx
+++ b/Accor_Ibis_Jaipur_Price_History.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -763,6 +763,296 @@
         </is>
       </c>
       <c r="L6" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-09-06 18:09:52</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-12-25</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-12-26</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>ibis Jaipur City Centre</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>STANDARD QUEEN ROOM</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>6270</v>
+      </c>
+      <c r="G7" t="n">
+        <v>6600</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>FLEXIBLE RATE</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>EUROPEAN_PLAN</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Cancel free of charge until 24th Dec 11:59 pm</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>No prepayment required</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-09-06 18:09:52</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-12-25</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2026-12-26</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>ibis Jaipur City Centre</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>STANDARD TWIN ROOM</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>6270</v>
+      </c>
+      <c r="G8" t="n">
+        <v>6600</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>FLEXIBLE RATE</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>EUROPEAN_PLAN</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Cancel free of charge until 24th Dec 11:59 pm</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>No prepayment required</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-09-06 18:09:52</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-12-25</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-12-26</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>ibis Jaipur City Centre</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Superior Queen Room - 30% discount on F&amp;B</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>6888</v>
+      </c>
+      <c r="G9" t="n">
+        <v>7250</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>FLEXIBLE RATE</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>EUROPEAN_PLAN</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Cancel free of charge until 24th Dec 11:59 pm</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>No prepayment required</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09-06 18:09:52</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-12-25</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2026-12-26</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>ibis Jaipur City Centre</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Superior Twin Room - 30% discount on F&amp;B</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>6888</v>
+      </c>
+      <c r="G10" t="n">
+        <v>7250</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>FLEXIBLE RATE</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>EUROPEAN_PLAN</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Cancel free of charge until 24th Dec 11:59 pm</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>No prepayment required</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-09-06 18:09:52</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-12-25</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2026-12-26</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>ibis Jaipur City Centre</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Family Retreat Room - 20% Off Spa</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>7220</v>
+      </c>
+      <c r="G11" t="n">
+        <v>7600</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>FLEXIBLE RATE</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>EUROPEAN_PLAN</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Cancel free of charge until 24th Dec 11:59 pm</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>No prepayment required</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
         <is>
           <t>YES</t>
         </is>

</xml_diff>